<commit_message>
feat(pinterest): publish batch of 12 public pins to live boards and sync trackers
</commit_message>
<xml_diff>
--- a/worksheets-tracker.xlsx
+++ b/worksheets-tracker.xlsx
@@ -653,12 +653,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1127096244305805491</t>
+          <t>1127096244305807423</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -725,12 +725,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1127096244305805487</t>
+          <t>1127096244305807418</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -797,12 +797,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1127096244305805483</t>
+          <t>1127096244305807413</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -869,12 +869,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1127096244305805475</t>
+          <t>1127096244305807408</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Nepali Worksheets</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1127096244305805470</t>
+          <t>1127096244305807405</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Nepali Worksheets</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1013,12 +1013,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1127096244305805468</t>
+          <t>1127096244305807402</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1127096244305805465</t>
+          <t>1127096244305807399</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1127096244305805460</t>
+          <t>1127096244305807396</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Nepali Worksheets</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1229,12 +1229,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1127096244305805456</t>
+          <t>1127096244305807392</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Nepali Worksheets</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1301,12 +1301,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1127096244305805448</t>
+          <t>1127096244305807387</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1373,12 +1373,12 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1127096244305805441</t>
+          <t>1127096244305807382</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1445,12 +1445,12 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1127096244305805215</t>
+          <t>1127096244305807324</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">

</xml_diff>

<commit_message>
feat(pinterest): sync 102 newly published public pins to tracking files and uploader
</commit_message>
<xml_diff>
--- a/worksheets-tracker.xlsx
+++ b/worksheets-tracker.xlsx
@@ -27005,17 +27005,17 @@
       </c>
       <c r="L368" t="inlineStr">
         <is>
-          <t>1127096244304350474</t>
+          <t>1127096244305808880</t>
         </is>
       </c>
       <c r="M368" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N368" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27077,17 +27077,17 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>1127096244304350484</t>
+          <t>1127096244305808883</t>
         </is>
       </c>
       <c r="M369" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N369" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27149,17 +27149,17 @@
       </c>
       <c r="L370" t="inlineStr">
         <is>
-          <t>1127096244304350488</t>
+          <t>1127096244305808885</t>
         </is>
       </c>
       <c r="M370" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N370" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27221,17 +27221,17 @@
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>1127096244304350497</t>
+          <t>1127096244305808888</t>
         </is>
       </c>
       <c r="M371" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N371" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27293,17 +27293,17 @@
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t>1127096244304350507</t>
+          <t>1127096244305808891</t>
         </is>
       </c>
       <c r="M372" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N372" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27365,17 +27365,17 @@
       </c>
       <c r="L373" t="inlineStr">
         <is>
-          <t>1127096244304350512</t>
+          <t>1127096244305808893</t>
         </is>
       </c>
       <c r="M373" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N373" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27437,17 +27437,17 @@
       </c>
       <c r="L374" t="inlineStr">
         <is>
-          <t>1127096244304350520</t>
+          <t>1127096244305808896</t>
         </is>
       </c>
       <c r="M374" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N374" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27509,17 +27509,17 @@
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t>1127096244304350527</t>
+          <t>1127096244305808900</t>
         </is>
       </c>
       <c r="M375" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N375" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27581,17 +27581,17 @@
       </c>
       <c r="L376" t="inlineStr">
         <is>
-          <t>1127096244304350530</t>
+          <t>1127096244305808902</t>
         </is>
       </c>
       <c r="M376" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N376" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27653,17 +27653,17 @@
       </c>
       <c r="L377" t="inlineStr">
         <is>
-          <t>1127096244304350536</t>
+          <t>1127096244305808905</t>
         </is>
       </c>
       <c r="M377" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N377" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27725,17 +27725,17 @@
       </c>
       <c r="L378" t="inlineStr">
         <is>
-          <t>1127096244304350541</t>
+          <t>1127096244305808911</t>
         </is>
       </c>
       <c r="M378" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N378" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27797,17 +27797,17 @@
       </c>
       <c r="L379" t="inlineStr">
         <is>
-          <t>1127096244304350547</t>
+          <t>1127096244305808915</t>
         </is>
       </c>
       <c r="M379" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N379" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -27869,17 +27869,17 @@
       </c>
       <c r="L380" t="inlineStr">
         <is>
-          <t>1127096244304350551</t>
+          <t>1127096244305808918</t>
         </is>
       </c>
       <c r="M380" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N380" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28013,17 +28013,17 @@
       </c>
       <c r="L382" t="inlineStr">
         <is>
-          <t>1127096244304350554</t>
+          <t>1127096244305808921</t>
         </is>
       </c>
       <c r="M382" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N382" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28085,17 +28085,17 @@
       </c>
       <c r="L383" t="inlineStr">
         <is>
-          <t>1127096244304350561</t>
+          <t>1127096244305808927</t>
         </is>
       </c>
       <c r="M383" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N383" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28157,17 +28157,17 @@
       </c>
       <c r="L384" t="inlineStr">
         <is>
-          <t>1127096244304350566</t>
+          <t>1127096244305808932</t>
         </is>
       </c>
       <c r="M384" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N384" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28229,17 +28229,17 @@
       </c>
       <c r="L385" t="inlineStr">
         <is>
-          <t>1127096244304350570</t>
+          <t>1127096244305808952</t>
         </is>
       </c>
       <c r="M385" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N385" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28373,17 +28373,17 @@
       </c>
       <c r="L387" t="inlineStr">
         <is>
-          <t>1127096244304350576</t>
+          <t>1127096244305808964</t>
         </is>
       </c>
       <c r="M387" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N387" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28445,17 +28445,17 @@
       </c>
       <c r="L388" t="inlineStr">
         <is>
-          <t>1127096244304350578</t>
+          <t>1127096244305808967</t>
         </is>
       </c>
       <c r="M388" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N388" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28517,17 +28517,17 @@
       </c>
       <c r="L389" t="inlineStr">
         <is>
-          <t>1127096244304350582</t>
+          <t>1127096244305808975</t>
         </is>
       </c>
       <c r="M389" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N389" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28589,17 +28589,17 @@
       </c>
       <c r="L390" t="inlineStr">
         <is>
-          <t>1127096244304350584</t>
+          <t>1127096244305808979</t>
         </is>
       </c>
       <c r="M390" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N390" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28661,17 +28661,17 @@
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>1127096244304350586</t>
+          <t>1127096244305808985</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N391" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28733,17 +28733,17 @@
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t>1127096244304350590</t>
+          <t>1127096244305808993</t>
         </is>
       </c>
       <c r="M392" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N392" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -28949,17 +28949,17 @@
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t>1127096244304350594</t>
+          <t>1127096244305809003</t>
         </is>
       </c>
       <c r="M395" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N395" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29021,17 +29021,17 @@
       </c>
       <c r="L396" t="inlineStr">
         <is>
-          <t>1127096244304350600</t>
+          <t>1127096244305809010</t>
         </is>
       </c>
       <c r="M396" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N396" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29093,17 +29093,17 @@
       </c>
       <c r="L397" t="inlineStr">
         <is>
-          <t>1127096244304350604</t>
+          <t>1127096244305809013</t>
         </is>
       </c>
       <c r="M397" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N397" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29165,17 +29165,17 @@
       </c>
       <c r="L398" t="inlineStr">
         <is>
-          <t>1127096244304350609</t>
+          <t>1127096244305809015</t>
         </is>
       </c>
       <c r="M398" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N398" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29237,17 +29237,17 @@
       </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t>1127096244304350616</t>
+          <t>1127096244305809018</t>
         </is>
       </c>
       <c r="M399" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N399" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29309,17 +29309,17 @@
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t>1127096244304350619</t>
+          <t>1127096244305809020</t>
         </is>
       </c>
       <c r="M400" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N400" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29381,17 +29381,17 @@
       </c>
       <c r="L401" t="inlineStr">
         <is>
-          <t>1127096244304350625</t>
+          <t>1127096244305809024</t>
         </is>
       </c>
       <c r="M401" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N401" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29525,17 +29525,17 @@
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t>1127096244304350634</t>
+          <t>1127096244305809029</t>
         </is>
       </c>
       <c r="M403" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N403" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29597,17 +29597,17 @@
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t>1127096244304350641</t>
+          <t>1127096244305809033</t>
         </is>
       </c>
       <c r="M404" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N404" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29669,17 +29669,17 @@
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t>1127096244304350646</t>
+          <t>1127096244305809037</t>
         </is>
       </c>
       <c r="M405" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N405" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29741,17 +29741,17 @@
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t>1127096244304350650</t>
+          <t>1127096244305809038</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N406" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29813,17 +29813,17 @@
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>1127096244304350656</t>
+          <t>1127096244305809041</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N407" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29885,17 +29885,17 @@
       </c>
       <c r="L408" t="inlineStr">
         <is>
-          <t>1127096244304350664</t>
+          <t>1127096244305809049</t>
         </is>
       </c>
       <c r="M408" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N408" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -29957,17 +29957,17 @@
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t>1127096244304350671</t>
+          <t>1127096244305809105</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N409" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30029,17 +30029,17 @@
       </c>
       <c r="L410" t="inlineStr">
         <is>
-          <t>1127096244304350681</t>
+          <t>1127096244305809136</t>
         </is>
       </c>
       <c r="M410" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N410" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30101,17 +30101,17 @@
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t>1127096244304350685</t>
+          <t>1127096244305809184</t>
         </is>
       </c>
       <c r="M411" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N411" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30173,17 +30173,17 @@
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t>1127096244304350691</t>
+          <t>1127096244305809208</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N412" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30245,17 +30245,17 @@
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t>1127096244304350695</t>
+          <t>1127096244305809247</t>
         </is>
       </c>
       <c r="M413" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N413" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30317,17 +30317,17 @@
       </c>
       <c r="L414" t="inlineStr">
         <is>
-          <t>1127096244304350701</t>
+          <t>1127096244305809275</t>
         </is>
       </c>
       <c r="M414" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N414" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30461,17 +30461,17 @@
       </c>
       <c r="L416" t="inlineStr">
         <is>
-          <t>1127096244304350706</t>
+          <t>1127096244305809307</t>
         </is>
       </c>
       <c r="M416" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N416" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30533,17 +30533,17 @@
       </c>
       <c r="L417" t="inlineStr">
         <is>
-          <t>1127096244304350710</t>
+          <t>1127096244305809345</t>
         </is>
       </c>
       <c r="M417" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N417" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30605,17 +30605,17 @@
       </c>
       <c r="L418" t="inlineStr">
         <is>
-          <t>1127096244304350717</t>
+          <t>1127096244305809364</t>
         </is>
       </c>
       <c r="M418" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N418" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30677,17 +30677,17 @@
       </c>
       <c r="L419" t="inlineStr">
         <is>
-          <t>1127096244304350721</t>
+          <t>1127096244305809446</t>
         </is>
       </c>
       <c r="M419" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N419" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30821,17 +30821,17 @@
       </c>
       <c r="L421" t="inlineStr">
         <is>
-          <t>1127096244304350729</t>
+          <t>1127096244305809482</t>
         </is>
       </c>
       <c r="M421" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N421" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30893,17 +30893,17 @@
       </c>
       <c r="L422" t="inlineStr">
         <is>
-          <t>1127096244304350734</t>
+          <t>1127096244305809508</t>
         </is>
       </c>
       <c r="M422" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N422" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -30965,17 +30965,17 @@
       </c>
       <c r="L423" t="inlineStr">
         <is>
-          <t>1127096244304350741</t>
+          <t>1127096244305809529</t>
         </is>
       </c>
       <c r="M423" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N423" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -31037,17 +31037,17 @@
       </c>
       <c r="L424" t="inlineStr">
         <is>
-          <t>1127096244304350755</t>
+          <t>1127096244305809563</t>
         </is>
       </c>
       <c r="M424" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N424" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -38957,17 +38957,17 @@
       </c>
       <c r="L534" t="inlineStr">
         <is>
-          <t>1127096244304351162</t>
+          <t>1127096244305808875</t>
         </is>
       </c>
       <c r="M534" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N534" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39029,17 +39029,17 @@
       </c>
       <c r="L535" t="inlineStr">
         <is>
-          <t>1127096244304351167</t>
+          <t>1127096244305808867</t>
         </is>
       </c>
       <c r="M535" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N535" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39101,17 +39101,17 @@
       </c>
       <c r="L536" t="inlineStr">
         <is>
-          <t>1127096244304351171</t>
+          <t>1127096244305808864</t>
         </is>
       </c>
       <c r="M536" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N536" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39173,17 +39173,17 @@
       </c>
       <c r="L537" t="inlineStr">
         <is>
-          <t>1127096244304351176</t>
+          <t>1127096244305808861</t>
         </is>
       </c>
       <c r="M537" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N537" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39245,17 +39245,17 @@
       </c>
       <c r="L538" t="inlineStr">
         <is>
-          <t>1127096244304351181</t>
+          <t>1127096244305808860</t>
         </is>
       </c>
       <c r="M538" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N538" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39317,17 +39317,17 @@
       </c>
       <c r="L539" t="inlineStr">
         <is>
-          <t>1127096244304351184</t>
+          <t>1127096244305808857</t>
         </is>
       </c>
       <c r="M539" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N539" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39389,17 +39389,17 @@
       </c>
       <c r="L540" t="inlineStr">
         <is>
-          <t>1127096244304351191</t>
+          <t>1127096244305808853</t>
         </is>
       </c>
       <c r="M540" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N540" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39461,17 +39461,17 @@
       </c>
       <c r="L541" t="inlineStr">
         <is>
-          <t>1127096244304351193</t>
+          <t>1127096244305808849</t>
         </is>
       </c>
       <c r="M541" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N541" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39533,17 +39533,17 @@
       </c>
       <c r="L542" t="inlineStr">
         <is>
-          <t>1127096244304351199</t>
+          <t>1127096244305808843</t>
         </is>
       </c>
       <c r="M542" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N542" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39605,17 +39605,17 @@
       </c>
       <c r="L543" t="inlineStr">
         <is>
-          <t>1127096244304351205</t>
+          <t>1127096244305808837</t>
         </is>
       </c>
       <c r="M543" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N543" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39677,17 +39677,17 @@
       </c>
       <c r="L544" t="inlineStr">
         <is>
-          <t>1127096244304351217</t>
+          <t>1127096244305808836</t>
         </is>
       </c>
       <c r="M544" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N544" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39749,17 +39749,17 @@
       </c>
       <c r="L545" t="inlineStr">
         <is>
-          <t>1127096244304351223</t>
+          <t>1127096244305808830</t>
         </is>
       </c>
       <c r="M545" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N545" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39821,17 +39821,17 @@
       </c>
       <c r="L546" t="inlineStr">
         <is>
-          <t>1127096244304351227</t>
+          <t>1127096244305808826</t>
         </is>
       </c>
       <c r="M546" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N546" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39893,17 +39893,17 @@
       </c>
       <c r="L547" t="inlineStr">
         <is>
-          <t>1127096244304351233</t>
+          <t>1127096244305808822</t>
         </is>
       </c>
       <c r="M547" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N547" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -39965,17 +39965,17 @@
       </c>
       <c r="L548" t="inlineStr">
         <is>
-          <t>1127096244304351237</t>
+          <t>1127096244305808815</t>
         </is>
       </c>
       <c r="M548" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N548" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40037,17 +40037,17 @@
       </c>
       <c r="L549" t="inlineStr">
         <is>
-          <t>1127096244304351241</t>
+          <t>1127096244305808805</t>
         </is>
       </c>
       <c r="M549" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N549" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40109,17 +40109,17 @@
       </c>
       <c r="L550" t="inlineStr">
         <is>
-          <t>1127096244304351247</t>
+          <t>1127096244305808801</t>
         </is>
       </c>
       <c r="M550" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N550" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40181,17 +40181,17 @@
       </c>
       <c r="L551" t="inlineStr">
         <is>
-          <t>1127096244304351254</t>
+          <t>1127096244305808796</t>
         </is>
       </c>
       <c r="M551" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N551" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40253,17 +40253,17 @@
       </c>
       <c r="L552" t="inlineStr">
         <is>
-          <t>1127096244304351257</t>
+          <t>1127096244305808790</t>
         </is>
       </c>
       <c r="M552" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N552" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40325,17 +40325,17 @@
       </c>
       <c r="L553" t="inlineStr">
         <is>
-          <t>1127096244304351264</t>
+          <t>1127096244305808783</t>
         </is>
       </c>
       <c r="M553" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N553" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40397,17 +40397,17 @@
       </c>
       <c r="L554" t="inlineStr">
         <is>
-          <t>1127096244304351269</t>
+          <t>1127096244305808774</t>
         </is>
       </c>
       <c r="M554" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N554" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40469,17 +40469,17 @@
       </c>
       <c r="L555" t="inlineStr">
         <is>
-          <t>1127096244304351273</t>
+          <t>1127096244305808770</t>
         </is>
       </c>
       <c r="M555" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N555" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40541,17 +40541,17 @@
       </c>
       <c r="L556" t="inlineStr">
         <is>
-          <t>1127096244304351280</t>
+          <t>1127096244305808766</t>
         </is>
       </c>
       <c r="M556" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N556" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40613,17 +40613,17 @@
       </c>
       <c r="L557" t="inlineStr">
         <is>
-          <t>1127096244304351288</t>
+          <t>1127096244305808761</t>
         </is>
       </c>
       <c r="M557" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N557" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40685,17 +40685,17 @@
       </c>
       <c r="L558" t="inlineStr">
         <is>
-          <t>1127096244304351295</t>
+          <t>1127096244305808757</t>
         </is>
       </c>
       <c r="M558" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N558" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40757,17 +40757,17 @@
       </c>
       <c r="L559" t="inlineStr">
         <is>
-          <t>1127096244304351298</t>
+          <t>1127096244305808753</t>
         </is>
       </c>
       <c r="M559" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N559" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40829,17 +40829,17 @@
       </c>
       <c r="L560" t="inlineStr">
         <is>
-          <t>1127096244304351304</t>
+          <t>1127096244305808749</t>
         </is>
       </c>
       <c r="M560" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N560" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40901,17 +40901,17 @@
       </c>
       <c r="L561" t="inlineStr">
         <is>
-          <t>1127096244304351309</t>
+          <t>1127096244305808744</t>
         </is>
       </c>
       <c r="M561" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N561" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -40973,17 +40973,17 @@
       </c>
       <c r="L562" t="inlineStr">
         <is>
-          <t>1127096244304351315</t>
+          <t>1127096244305808739</t>
         </is>
       </c>
       <c r="M562" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N562" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41045,17 +41045,17 @@
       </c>
       <c r="L563" t="inlineStr">
         <is>
-          <t>1127096244304351317</t>
+          <t>1127096244305808734</t>
         </is>
       </c>
       <c r="M563" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N563" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41117,17 +41117,17 @@
       </c>
       <c r="L564" t="inlineStr">
         <is>
-          <t>1127096244304351321</t>
+          <t>1127096244305808729</t>
         </is>
       </c>
       <c r="M564" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N564" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41189,17 +41189,17 @@
       </c>
       <c r="L565" t="inlineStr">
         <is>
-          <t>1127096244304351328</t>
+          <t>1127096244305808726</t>
         </is>
       </c>
       <c r="M565" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N565" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41261,17 +41261,17 @@
       </c>
       <c r="L566" t="inlineStr">
         <is>
-          <t>1127096244304351342</t>
+          <t>1127096244305808719</t>
         </is>
       </c>
       <c r="M566" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N566" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41333,17 +41333,17 @@
       </c>
       <c r="L567" t="inlineStr">
         <is>
-          <t>1127096244304351348</t>
+          <t>1127096244305808713</t>
         </is>
       </c>
       <c r="M567" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N567" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41405,17 +41405,17 @@
       </c>
       <c r="L568" t="inlineStr">
         <is>
-          <t>1127096244304351353</t>
+          <t>1127096244305808702</t>
         </is>
       </c>
       <c r="M568" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N568" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41477,17 +41477,17 @@
       </c>
       <c r="L569" t="inlineStr">
         <is>
-          <t>1127096244304351358</t>
+          <t>1127096244305808695</t>
         </is>
       </c>
       <c r="M569" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N569" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41549,17 +41549,17 @@
       </c>
       <c r="L570" t="inlineStr">
         <is>
-          <t>1127096244304351369</t>
+          <t>1127096244305808691</t>
         </is>
       </c>
       <c r="M570" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N570" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41621,17 +41621,17 @@
       </c>
       <c r="L571" t="inlineStr">
         <is>
-          <t>1127096244304351375</t>
+          <t>1127096244305808685</t>
         </is>
       </c>
       <c r="M571" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N571" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41693,17 +41693,17 @@
       </c>
       <c r="L572" t="inlineStr">
         <is>
-          <t>1127096244304351379</t>
+          <t>1127096244305808682</t>
         </is>
       </c>
       <c r="M572" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N572" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41765,17 +41765,17 @@
       </c>
       <c r="L573" t="inlineStr">
         <is>
-          <t>1127096244304351385</t>
+          <t>1127096244305808678</t>
         </is>
       </c>
       <c r="M573" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N573" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41837,17 +41837,17 @@
       </c>
       <c r="L574" t="inlineStr">
         <is>
-          <t>1127096244304351391</t>
+          <t>1127096244305808673</t>
         </is>
       </c>
       <c r="M574" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N574" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41909,17 +41909,17 @@
       </c>
       <c r="L575" t="inlineStr">
         <is>
-          <t>1127096244304351398</t>
+          <t>1127096244305808666</t>
         </is>
       </c>
       <c r="M575" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N575" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -41981,17 +41981,17 @@
       </c>
       <c r="L576" t="inlineStr">
         <is>
-          <t>1127096244304351409</t>
+          <t>1127096244305808659</t>
         </is>
       </c>
       <c r="M576" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N576" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42053,17 +42053,17 @@
       </c>
       <c r="L577" t="inlineStr">
         <is>
-          <t>1127096244304351416</t>
+          <t>1127096244305808652</t>
         </is>
       </c>
       <c r="M577" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N577" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42125,17 +42125,17 @@
       </c>
       <c r="L578" t="inlineStr">
         <is>
-          <t>1127096244304351424</t>
+          <t>1127096244305808646</t>
         </is>
       </c>
       <c r="M578" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N578" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42197,17 +42197,17 @@
       </c>
       <c r="L579" t="inlineStr">
         <is>
-          <t>1127096244304351433</t>
+          <t>1127096244305808643</t>
         </is>
       </c>
       <c r="M579" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N579" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42269,17 +42269,17 @@
       </c>
       <c r="L580" t="inlineStr">
         <is>
-          <t>1127096244304351443</t>
+          <t>1127096244305808641</t>
         </is>
       </c>
       <c r="M580" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N580" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42341,17 +42341,17 @@
       </c>
       <c r="L581" t="inlineStr">
         <is>
-          <t>1127096244304351449</t>
+          <t>1127096244305808639</t>
         </is>
       </c>
       <c r="M581" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N581" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42413,17 +42413,17 @@
       </c>
       <c r="L582" t="inlineStr">
         <is>
-          <t>1127096244304351458</t>
+          <t>1127096244305808631</t>
         </is>
       </c>
       <c r="M582" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N582" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42485,17 +42485,17 @@
       </c>
       <c r="L583" t="inlineStr">
         <is>
-          <t>1127096244304351465</t>
+          <t>1127096244305808625</t>
         </is>
       </c>
       <c r="M583" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N583" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42557,17 +42557,17 @@
       </c>
       <c r="L584" t="inlineStr">
         <is>
-          <t>1127096244304351474</t>
+          <t>1127096244305808617</t>
         </is>
       </c>
       <c r="M584" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N584" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -42629,17 +42629,17 @@
       </c>
       <c r="L585" t="inlineStr">
         <is>
-          <t>1127096244304351480</t>
+          <t>1127096244305808611</t>
         </is>
       </c>
       <c r="M585" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N585" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(pinterest): sync 94 newly published public pins to tracking files and uploader
</commit_message>
<xml_diff>
--- a/worksheets-tracker.xlsx
+++ b/worksheets-tracker.xlsx
@@ -11525,17 +11525,17 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>1127096244304349471</t>
+          <t>1127096244305969079</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -11597,17 +11597,17 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>1127096244304349473</t>
+          <t>1127096244305969085</t>
         </is>
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -11669,17 +11669,17 @@
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>1127096244304349476</t>
+          <t>1127096244305969088</t>
         </is>
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -11741,17 +11741,17 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>1127096244304349481</t>
+          <t>1127096244305969093</t>
         </is>
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -11813,17 +11813,17 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>1127096244304349482</t>
+          <t>1127096244305969097</t>
         </is>
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12245,17 +12245,17 @@
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>1127096244304349505</t>
+          <t>1127096244305969098</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12317,17 +12317,17 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>1127096244304349513</t>
+          <t>1127096244305969104</t>
         </is>
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12389,17 +12389,17 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>1127096244304349516</t>
+          <t>1127096244305969117</t>
         </is>
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12461,17 +12461,17 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>1127096244304349518</t>
+          <t>1127096244305969121</t>
         </is>
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12533,17 +12533,17 @@
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>1127096244304349523</t>
+          <t>1127096244305969127</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12605,17 +12605,17 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>1127096244304349528</t>
+          <t>1127096244305969131</t>
         </is>
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12677,17 +12677,17 @@
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>1127096244304349534</t>
+          <t>1127096244305969139</t>
         </is>
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12749,17 +12749,17 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>1127096244304349535</t>
+          <t>1127096244305969142</t>
         </is>
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12821,17 +12821,17 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>1127096244304349538</t>
+          <t>1127096244305969145</t>
         </is>
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12893,17 +12893,17 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>1127096244304349541</t>
+          <t>1127096244305969153</t>
         </is>
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -12965,17 +12965,17 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>1127096244304349545</t>
+          <t>1127096244305969155</t>
         </is>
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13037,17 +13037,17 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>1127096244304349550</t>
+          <t>1127096244305969156</t>
         </is>
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13109,17 +13109,17 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>1127096244304349553</t>
+          <t>1127096244305969159</t>
         </is>
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13181,17 +13181,17 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>1127096244304349556</t>
+          <t>1127096244305969162</t>
         </is>
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13253,17 +13253,17 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>1127096244304349557</t>
+          <t>1127096244305969166</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13325,17 +13325,17 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>1127096244304349561</t>
+          <t>1127096244305969168</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13397,17 +13397,17 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>1127096244304349564</t>
+          <t>1127096244305969171</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13469,17 +13469,17 @@
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>1127096244304349565</t>
+          <t>1127096244305969176</t>
         </is>
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13613,17 +13613,17 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>1127096244304349568</t>
+          <t>1127096244305969182</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13685,17 +13685,17 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>1127096244304349571</t>
+          <t>1127096244305969186</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13757,17 +13757,17 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>1127096244304349580</t>
+          <t>1127096244305969190</t>
         </is>
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13829,17 +13829,17 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>1127096244304349585</t>
+          <t>1127096244305969194</t>
         </is>
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13901,17 +13901,17 @@
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t>1127096244304349590</t>
+          <t>1127096244305969201</t>
         </is>
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -13973,17 +13973,17 @@
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t>1127096244304349592</t>
+          <t>1127096244305969204</t>
         </is>
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14045,17 +14045,17 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>1127096244304349598</t>
+          <t>1127096244305969205</t>
         </is>
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14117,17 +14117,17 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>1127096244304349600</t>
+          <t>1127096244305969209</t>
         </is>
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14189,17 +14189,17 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>1127096244304349607</t>
+          <t>1127096244305969219</t>
         </is>
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14261,17 +14261,17 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>1127096244304349611</t>
+          <t>1127096244305969223</t>
         </is>
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14333,17 +14333,17 @@
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>1127096244304349617</t>
+          <t>1127096244305969224</t>
         </is>
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14405,17 +14405,17 @@
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>1127096244304349628</t>
+          <t>1127096244305969228</t>
         </is>
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14477,17 +14477,17 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>1127096244304349632</t>
+          <t>1127096244305969232</t>
         </is>
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14549,17 +14549,17 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>1127096244304349641</t>
+          <t>1127096244305969240</t>
         </is>
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14621,17 +14621,17 @@
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>1127096244304349643</t>
+          <t>1127096244305969244</t>
         </is>
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14693,17 +14693,17 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>1127096244304349647</t>
+          <t>1127096244305969247</t>
         </is>
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14837,17 +14837,17 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>1127096244304349650</t>
+          <t>1127096244305969250</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14909,17 +14909,17 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>1127096244304349654</t>
+          <t>1127096244305969254</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -14981,17 +14981,17 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>1127096244304349656</t>
+          <t>1127096244305969255</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15053,17 +15053,17 @@
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>1127096244304349659</t>
+          <t>1127096244305969258</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N202" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15125,17 +15125,17 @@
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>1127096244304349665</t>
+          <t>1127096244305969261</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N203" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15197,17 +15197,17 @@
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t>1127096244304349669</t>
+          <t>1127096244305969266</t>
         </is>
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15269,17 +15269,17 @@
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>1127096244304349676</t>
+          <t>1127096244305969271</t>
         </is>
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15341,17 +15341,17 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>1127096244304349679</t>
+          <t>1127096244305969277</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15413,17 +15413,17 @@
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t>1127096244304349683</t>
+          <t>1127096244305969282</t>
         </is>
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N207" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15485,17 +15485,17 @@
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>1127096244304349685</t>
+          <t>1127096244305969285</t>
         </is>
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N208" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15557,17 +15557,17 @@
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>1127096244304349688</t>
+          <t>1127096244305969288</t>
         </is>
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N209" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15629,17 +15629,17 @@
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t>1127096244304349694</t>
+          <t>1127096244305969290</t>
         </is>
       </c>
       <c r="M210" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15701,17 +15701,17 @@
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>1127096244304349698</t>
+          <t>1127096244305969294</t>
         </is>
       </c>
       <c r="M211" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N211" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15773,17 +15773,17 @@
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t>1127096244304349703</t>
+          <t>1127096244305969295</t>
         </is>
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -15917,17 +15917,17 @@
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t>1127096244304349713</t>
+          <t>1127096244305969298</t>
         </is>
       </c>
       <c r="M214" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16061,17 +16061,17 @@
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t>1127096244304349722</t>
+          <t>1127096244305969304</t>
         </is>
       </c>
       <c r="M216" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16277,17 +16277,17 @@
       </c>
       <c r="L219" t="inlineStr">
         <is>
-          <t>1127096244304349735</t>
+          <t>1127096244305969305</t>
         </is>
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N219" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16421,17 +16421,17 @@
       </c>
       <c r="L221" t="inlineStr">
         <is>
-          <t>1127096244304349748</t>
+          <t>1127096244305969306</t>
         </is>
       </c>
       <c r="M221" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N221" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16565,17 +16565,17 @@
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>1127096244304349754</t>
+          <t>1127096244305969308</t>
         </is>
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N223" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16637,17 +16637,17 @@
       </c>
       <c r="L224" t="inlineStr">
         <is>
-          <t>1127096244304349762</t>
+          <t>1127096244305969312</t>
         </is>
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N224" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16709,17 +16709,17 @@
       </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t>1127096244304349765</t>
+          <t>1127096244305969315</t>
         </is>
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N225" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16781,17 +16781,17 @@
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>1127096244304349768</t>
+          <t>1127096244305969318</t>
         </is>
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N226" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16853,17 +16853,17 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>1127096244304349773</t>
+          <t>1127096244305969320</t>
         </is>
       </c>
       <c r="M227" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N227" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16925,17 +16925,17 @@
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>1127096244304349776</t>
+          <t>1127096244305969322</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N228" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -16997,17 +16997,17 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>1127096244304349777</t>
+          <t>1127096244305969324</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N229" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -17069,17 +17069,17 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>1127096244304349784</t>
+          <t>1127096244305969326</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N230" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -17285,17 +17285,17 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>1127096244304349795</t>
+          <t>1127096244305969327</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N233" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -17429,17 +17429,17 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>1127096244304349803</t>
+          <t>1127096244305969332</t>
         </is>
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -17861,17 +17861,17 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>1127096244304349820</t>
+          <t>1127096244305969334</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -17933,17 +17933,17 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>1127096244304349823</t>
+          <t>1127096244305969337</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18077,17 +18077,17 @@
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>1127096244304349834</t>
+          <t>1127096244305969345</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18149,17 +18149,17 @@
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>1127096244304349836</t>
+          <t>1127096244305969351</t>
         </is>
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18221,17 +18221,17 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>1127096244304349845</t>
+          <t>1127096244305969355</t>
         </is>
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18293,17 +18293,17 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>1127096244304349848</t>
+          <t>1127096244305969359</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N247" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18365,17 +18365,17 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>1127096244304349853</t>
+          <t>1127096244305969362</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18437,17 +18437,17 @@
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>1127096244304349859</t>
+          <t>1127096244305969366</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N249" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18509,17 +18509,17 @@
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>1127096244304349864</t>
+          <t>1127096244305969369</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N250" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18581,17 +18581,17 @@
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>1127096244304349867</t>
+          <t>1127096244305969373</t>
         </is>
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N251" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18653,17 +18653,17 @@
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>1127096244304349872</t>
+          <t>1127096244305969379</t>
         </is>
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N252" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18725,17 +18725,17 @@
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>1127096244304349877</t>
+          <t>1127096244305969383</t>
         </is>
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N253" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18797,17 +18797,17 @@
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t>1127096244304349883</t>
+          <t>1127096244305969390</t>
         </is>
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N254" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18869,17 +18869,17 @@
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>1127096244304349885</t>
+          <t>1127096244305969392</t>
         </is>
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -18941,17 +18941,17 @@
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>1127096244304349895</t>
+          <t>1127096244305969396</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N256" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19013,17 +19013,17 @@
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>1127096244304349900</t>
+          <t>1127096244305969399</t>
         </is>
       </c>
       <c r="M257" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N257" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19085,17 +19085,17 @@
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>1127096244304349905</t>
+          <t>1127096244305969403</t>
         </is>
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N258" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19157,17 +19157,17 @@
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>1127096244304349913</t>
+          <t>1127096244305969407</t>
         </is>
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N259" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19229,17 +19229,17 @@
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>1127096244304349917</t>
+          <t>1127096244305969409</t>
         </is>
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N260" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19301,17 +19301,17 @@
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>1127096244304349921</t>
+          <t>1127096244305969415</t>
         </is>
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N261" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19373,17 +19373,17 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>1127096244304349928</t>
+          <t>1127096244305969416</t>
         </is>
       </c>
       <c r="M262" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N262" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19445,17 +19445,17 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>1127096244304349931</t>
+          <t>1127096244305969419</t>
         </is>
       </c>
       <c r="M263" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N263" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19517,17 +19517,17 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>1127096244304349935</t>
+          <t>1127096244305969422</t>
         </is>
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N264" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19589,17 +19589,17 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>1127096244304349939</t>
+          <t>1127096244305969426</t>
         </is>
       </c>
       <c r="M265" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N265" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19661,17 +19661,17 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>1127096244304349942</t>
+          <t>1127096244305969431</t>
         </is>
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N266" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19733,17 +19733,17 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>1127096244304349948</t>
+          <t>1127096244305969438</t>
         </is>
       </c>
       <c r="M267" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N267" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -19805,17 +19805,17 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>1127096244304349953</t>
+          <t>1127096244305969441</t>
         </is>
       </c>
       <c r="M268" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N268" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracking): mark Halloween worksheets 50046-50051 as Pinned
Pins posted to production board 'Fun Worksheets For Kids' via
the Pinterest connector (pin.py --prod). Pin IDs recorded in the
MD ledger, XLSX tracker, and Google Sheet.
</commit_message>
<xml_diff>
--- a/worksheets-tracker.xlsx
+++ b/worksheets-tracker.xlsx
@@ -648,22 +648,22 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Not pinned</t>
+          <t>Pinned</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1127096244306045986</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -720,22 +720,22 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Not pinned</t>
+          <t>Pinned</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1127096244306046019</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -792,22 +792,22 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Not pinned</t>
+          <t>Pinned</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1127096244306046045</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -864,22 +864,22 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Not pinned</t>
+          <t>Pinned</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1127096244306046066</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -936,22 +936,22 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Not pinned</t>
+          <t>Pinned</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1127096244306046093</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1008,22 +1008,22 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Not pinned</t>
+          <t>Pinned</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1127096244306046127</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(pinterest): sync 89 newly published public pins to tracking files and uploader
</commit_message>
<xml_diff>
--- a/worksheets-tracker.xlsx
+++ b/worksheets-tracker.xlsx
@@ -648,22 +648,22 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pinned</t>
+          <t>Not pinned</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1127096244306045986</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Fun Worksheets For Kids</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -720,22 +720,22 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Pinned</t>
+          <t>Not pinned</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1127096244306046019</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Fun Worksheets For Kids</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -792,22 +792,22 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pinned</t>
+          <t>Not pinned</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1127096244306046045</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Fun Worksheets For Kids</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -864,22 +864,22 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Pinned</t>
+          <t>Not pinned</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1127096244306046066</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Fun Worksheets For Kids</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -936,22 +936,22 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Pinned</t>
+          <t>Not pinned</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1127096244306046093</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Fun Worksheets For Kids</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1008,22 +1008,22 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Pinned</t>
+          <t>Not pinned</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1127096244306046127</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Fun Worksheets For Kids</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -20309,17 +20309,17 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>1127096244304349957</t>
+          <t>1127096244306046256</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N275" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20381,17 +20381,17 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>1127096244304349964</t>
+          <t>1127096244306046262</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N276" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20453,17 +20453,17 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>1127096244304349969</t>
+          <t>1127096244306046269</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N277" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20525,17 +20525,17 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>1127096244304349973</t>
+          <t>1127096244306046277</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N278" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20597,17 +20597,17 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>1127096244304349978</t>
+          <t>1127096244306046287</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N279" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20669,17 +20669,17 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>1127096244304349983</t>
+          <t>1127096244306046296</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N280" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20741,17 +20741,17 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>1127096244304349986</t>
+          <t>1127096244306046302</t>
         </is>
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N281" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20813,17 +20813,17 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>1127096244304349989</t>
+          <t>1127096244306046308</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N282" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20885,17 +20885,17 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>1127096244304350003</t>
+          <t>1127096244306046319</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -20957,17 +20957,17 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>1127096244304350011</t>
+          <t>1127096244306046323</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N284" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21029,17 +21029,17 @@
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>1127096244304350017</t>
+          <t>1127096244306046329</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N285" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21101,17 +21101,17 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>1127096244304350018</t>
+          <t>1127096244306046333</t>
         </is>
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N286" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21173,17 +21173,17 @@
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>1127096244304350023</t>
+          <t>1127096244306046338</t>
         </is>
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N287" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21245,17 +21245,17 @@
       </c>
       <c r="L288" t="inlineStr">
         <is>
-          <t>1127096244304350027</t>
+          <t>1127096244306046341</t>
         </is>
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N288" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21317,17 +21317,17 @@
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>1127096244304350033</t>
+          <t>1127096244306046349</t>
         </is>
       </c>
       <c r="M289" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N289" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21389,17 +21389,17 @@
       </c>
       <c r="L290" t="inlineStr">
         <is>
-          <t>1127096244304350044</t>
+          <t>1127096244306046356</t>
         </is>
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N290" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21461,17 +21461,17 @@
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t>1127096244304350046</t>
+          <t>1127096244306046360</t>
         </is>
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N291" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21533,17 +21533,17 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>1127096244304350051</t>
+          <t>1127096244306046366</t>
         </is>
       </c>
       <c r="M292" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N292" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21605,17 +21605,17 @@
       </c>
       <c r="L293" t="inlineStr">
         <is>
-          <t>1127096244304350057</t>
+          <t>1127096244306046373</t>
         </is>
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21677,17 +21677,17 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>1127096244304350066</t>
+          <t>1127096244306046377</t>
         </is>
       </c>
       <c r="M294" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N294" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21749,17 +21749,17 @@
       </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t>1127096244304350068</t>
+          <t>1127096244306046383</t>
         </is>
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N295" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21821,17 +21821,17 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>1127096244304350072</t>
+          <t>1127096244306046389</t>
         </is>
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N296" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21893,17 +21893,17 @@
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>1127096244304350083</t>
+          <t>1127096244306046397</t>
         </is>
       </c>
       <c r="M297" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N297" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -21965,17 +21965,17 @@
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t>1127096244304350089</t>
+          <t>1127096244306046401</t>
         </is>
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22037,17 +22037,17 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>1127096244304350092</t>
+          <t>1127096244306046407</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N299" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22109,17 +22109,17 @@
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t>1127096244304350096</t>
+          <t>1127096244306046415</t>
         </is>
       </c>
       <c r="M300" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N300" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22181,17 +22181,17 @@
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>1127096244304350099</t>
+          <t>1127096244306046420</t>
         </is>
       </c>
       <c r="M301" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N301" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22253,17 +22253,17 @@
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t>1127096244304350107</t>
+          <t>1127096244306046428</t>
         </is>
       </c>
       <c r="M302" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N302" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22325,17 +22325,17 @@
       </c>
       <c r="L303" t="inlineStr">
         <is>
-          <t>1127096244304350111</t>
+          <t>1127096244306046432</t>
         </is>
       </c>
       <c r="M303" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N303" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22397,17 +22397,17 @@
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t>1127096244304350117</t>
+          <t>1127096244306046435</t>
         </is>
       </c>
       <c r="M304" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N304" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22469,17 +22469,17 @@
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t>1127096244304350127</t>
+          <t>1127096244306046442</t>
         </is>
       </c>
       <c r="M305" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N305" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22541,17 +22541,17 @@
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t>1127096244304350130</t>
+          <t>1127096244306046446</t>
         </is>
       </c>
       <c r="M306" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N306" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22613,17 +22613,17 @@
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t>1127096244304350134</t>
+          <t>1127096244306046449</t>
         </is>
       </c>
       <c r="M307" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N307" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22685,17 +22685,17 @@
       </c>
       <c r="L308" t="inlineStr">
         <is>
-          <t>1127096244304350137</t>
+          <t>1127096244306046454</t>
         </is>
       </c>
       <c r="M308" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N308" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22757,17 +22757,17 @@
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t>1127096244304350138</t>
+          <t>1127096244306046458</t>
         </is>
       </c>
       <c r="M309" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N309" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22829,17 +22829,17 @@
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t>1127096244304350140</t>
+          <t>1127096244306046463</t>
         </is>
       </c>
       <c r="M310" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N310" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22901,17 +22901,17 @@
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>1127096244304350142</t>
+          <t>1127096244306046470</t>
         </is>
       </c>
       <c r="M311" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N311" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -22973,17 +22973,17 @@
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>1127096244304350146</t>
+          <t>1127096244306046474</t>
         </is>
       </c>
       <c r="M312" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N312" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23045,17 +23045,17 @@
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>1127096244304350151</t>
+          <t>1127096244306046476</t>
         </is>
       </c>
       <c r="M313" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N313" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23117,17 +23117,17 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>1127096244304350153</t>
+          <t>1127096244306046483</t>
         </is>
       </c>
       <c r="M314" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N314" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23189,17 +23189,17 @@
       </c>
       <c r="L315" t="inlineStr">
         <is>
-          <t>1127096244304350156</t>
+          <t>1127096244306046486</t>
         </is>
       </c>
       <c r="M315" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N315" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23261,17 +23261,17 @@
       </c>
       <c r="L316" t="inlineStr">
         <is>
-          <t>1127096244304350160</t>
+          <t>1127096244306046493</t>
         </is>
       </c>
       <c r="M316" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N316" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23333,17 +23333,17 @@
       </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>1127096244304350166</t>
+          <t>1127096244306046496</t>
         </is>
       </c>
       <c r="M317" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N317" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23405,17 +23405,17 @@
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t>1127096244304350175</t>
+          <t>1127096244306046501</t>
         </is>
       </c>
       <c r="M318" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N318" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23477,17 +23477,17 @@
       </c>
       <c r="L319" t="inlineStr">
         <is>
-          <t>1127096244304350181</t>
+          <t>1127096244306046504</t>
         </is>
       </c>
       <c r="M319" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N319" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23549,17 +23549,17 @@
       </c>
       <c r="L320" t="inlineStr">
         <is>
-          <t>1127096244304350185</t>
+          <t>1127096244306046513</t>
         </is>
       </c>
       <c r="M320" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N320" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23621,17 +23621,17 @@
       </c>
       <c r="L321" t="inlineStr">
         <is>
-          <t>1127096244304350194</t>
+          <t>1127096244306046518</t>
         </is>
       </c>
       <c r="M321" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N321" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23693,17 +23693,17 @@
       </c>
       <c r="L322" t="inlineStr">
         <is>
-          <t>1127096244304350202</t>
+          <t>1127096244306046524</t>
         </is>
       </c>
       <c r="M322" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N322" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23765,17 +23765,17 @@
       </c>
       <c r="L323" t="inlineStr">
         <is>
-          <t>1127096244304350206</t>
+          <t>1127096244306046528</t>
         </is>
       </c>
       <c r="M323" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N323" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23837,17 +23837,17 @@
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t>1127096244304350211</t>
+          <t>1127096244306046535</t>
         </is>
       </c>
       <c r="M324" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N324" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23909,17 +23909,17 @@
       </c>
       <c r="L325" t="inlineStr">
         <is>
-          <t>1127096244304350215</t>
+          <t>1127096244306046540</t>
         </is>
       </c>
       <c r="M325" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N325" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -23981,17 +23981,17 @@
       </c>
       <c r="L326" t="inlineStr">
         <is>
-          <t>1127096244304350220</t>
+          <t>1127096244306046548</t>
         </is>
       </c>
       <c r="M326" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N326" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24125,17 +24125,17 @@
       </c>
       <c r="L328" t="inlineStr">
         <is>
-          <t>1127096244304350224</t>
+          <t>1127096244306046551</t>
         </is>
       </c>
       <c r="M328" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N328" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24197,17 +24197,17 @@
       </c>
       <c r="L329" t="inlineStr">
         <is>
-          <t>1127096244304350228</t>
+          <t>1127096244306046555</t>
         </is>
       </c>
       <c r="M329" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N329" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24269,17 +24269,17 @@
       </c>
       <c r="L330" t="inlineStr">
         <is>
-          <t>1127096244304350231</t>
+          <t>1127096244306046561</t>
         </is>
       </c>
       <c r="M330" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N330" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24341,17 +24341,17 @@
       </c>
       <c r="L331" t="inlineStr">
         <is>
-          <t>1127096244304350235</t>
+          <t>1127096244306046563</t>
         </is>
       </c>
       <c r="M331" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N331" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24413,17 +24413,17 @@
       </c>
       <c r="L332" t="inlineStr">
         <is>
-          <t>1127096244304350241</t>
+          <t>1127096244306046568</t>
         </is>
       </c>
       <c r="M332" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N332" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24485,17 +24485,17 @@
       </c>
       <c r="L333" t="inlineStr">
         <is>
-          <t>1127096244304350244</t>
+          <t>1127096244306046572</t>
         </is>
       </c>
       <c r="M333" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N333" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24557,17 +24557,17 @@
       </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t>1127096244304350251</t>
+          <t>1127096244306046578</t>
         </is>
       </c>
       <c r="M334" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N334" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24629,17 +24629,17 @@
       </c>
       <c r="L335" t="inlineStr">
         <is>
-          <t>1127096244304350255</t>
+          <t>1127096244306046583</t>
         </is>
       </c>
       <c r="M335" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N335" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24701,17 +24701,17 @@
       </c>
       <c r="L336" t="inlineStr">
         <is>
-          <t>1127096244304350258</t>
+          <t>1127096244306046593</t>
         </is>
       </c>
       <c r="M336" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N336" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24773,17 +24773,17 @@
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t>1127096244304350264</t>
+          <t>1127096244306046601</t>
         </is>
       </c>
       <c r="M337" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N337" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24845,17 +24845,17 @@
       </c>
       <c r="L338" t="inlineStr">
         <is>
-          <t>1127096244304350267</t>
+          <t>1127096244306046607</t>
         </is>
       </c>
       <c r="M338" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N338" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24917,17 +24917,17 @@
       </c>
       <c r="L339" t="inlineStr">
         <is>
-          <t>1127096244304350274</t>
+          <t>1127096244306046611</t>
         </is>
       </c>
       <c r="M339" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N339" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -24989,17 +24989,17 @@
       </c>
       <c r="L340" t="inlineStr">
         <is>
-          <t>1127096244304350280</t>
+          <t>1127096244306046616</t>
         </is>
       </c>
       <c r="M340" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N340" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25061,17 +25061,17 @@
       </c>
       <c r="L341" t="inlineStr">
         <is>
-          <t>1127096244304350284</t>
+          <t>1127096244306046625</t>
         </is>
       </c>
       <c r="M341" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N341" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25133,17 +25133,17 @@
       </c>
       <c r="L342" t="inlineStr">
         <is>
-          <t>1127096244304350289</t>
+          <t>1127096244306046630</t>
         </is>
       </c>
       <c r="M342" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N342" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25205,17 +25205,17 @@
       </c>
       <c r="L343" t="inlineStr">
         <is>
-          <t>1127096244304350293</t>
+          <t>1127096244306046635</t>
         </is>
       </c>
       <c r="M343" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N343" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25277,17 +25277,17 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t>1127096244304350300</t>
+          <t>1127096244306046637</t>
         </is>
       </c>
       <c r="M344" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N344" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25421,17 +25421,17 @@
       </c>
       <c r="L346" t="inlineStr">
         <is>
-          <t>1127096244304350306</t>
+          <t>1127096244306046639</t>
         </is>
       </c>
       <c r="M346" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N346" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25493,17 +25493,17 @@
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t>1127096244304350310</t>
+          <t>1127096244306046642</t>
         </is>
       </c>
       <c r="M347" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N347" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25565,17 +25565,17 @@
       </c>
       <c r="L348" t="inlineStr">
         <is>
-          <t>1127096244304350313</t>
+          <t>1127096244306046649</t>
         </is>
       </c>
       <c r="M348" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N348" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25637,17 +25637,17 @@
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t>1127096244304350318</t>
+          <t>1127096244306046655</t>
         </is>
       </c>
       <c r="M349" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N349" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25709,17 +25709,17 @@
       </c>
       <c r="L350" t="inlineStr">
         <is>
-          <t>1127096244304350320</t>
+          <t>1127096244306046661</t>
         </is>
       </c>
       <c r="M350" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N350" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25781,17 +25781,17 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t>1127096244304350327</t>
+          <t>1127096244306046668</t>
         </is>
       </c>
       <c r="M351" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N351" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25853,17 +25853,17 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t>1127096244304350332</t>
+          <t>1127096244306046677</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N352" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25925,17 +25925,17 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t>1127096244304350337</t>
+          <t>1127096244306046686</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N353" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -25997,17 +25997,17 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t>1127096244304350341</t>
+          <t>1127096244306046688</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N354" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26141,17 +26141,17 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t>1127096244304350347</t>
+          <t>1127096244306046694</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N356" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26213,17 +26213,17 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t>1127096244304350349</t>
+          <t>1127096244306046699</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N357" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26285,17 +26285,17 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t>1127096244304350355</t>
+          <t>1127096244306046704</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N358" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26357,17 +26357,17 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t>1127096244304350362</t>
+          <t>1127096244306046710</t>
         </is>
       </c>
       <c r="M359" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N359" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26429,17 +26429,17 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t>1127096244304350371</t>
+          <t>1127096244306046715</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N360" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26501,17 +26501,17 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t>1127096244304350377</t>
+          <t>1127096244306046717</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N361" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26573,17 +26573,17 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>1127096244304350382</t>
+          <t>1127096244306046723</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N362" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26645,17 +26645,17 @@
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t>1127096244304350392</t>
+          <t>1127096244306046727</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N363" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -26717,17 +26717,17 @@
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>1127096244304350399</t>
+          <t>1127096244306046732</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N364" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -27005,17 +27005,17 @@
       </c>
       <c r="L368" t="inlineStr">
         <is>
-          <t>1127096244304350419</t>
+          <t>1127096244306046737</t>
         </is>
       </c>
       <c r="M368" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Fun Worksheets For Kids</t>
         </is>
       </c>
       <c r="N368" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -27149,17 +27149,17 @@
       </c>
       <c r="L370" t="inlineStr">
         <is>
-          <t>1127096244304350431</t>
+          <t>1127096244306046746</t>
         </is>
       </c>
       <c r="M370" t="inlineStr">
         <is>
-          <t>Sandbox Test Worksheets</t>
+          <t>Line Tracing Activities for PreSchool and Nursery</t>
         </is>
       </c>
       <c r="N370" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>

</xml_diff>